<commit_message>
Bestellliste: geprüfte Links Berrybase/Reichelt/openelab (16.10.), Lochraster-Ersatz
</commit_message>
<xml_diff>
--- a/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
+++ b/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amazon-Bestellliste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Andere Shops" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1902,4 +1903,717 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Teil</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Menge</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Einzelpreis €</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Summe €</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Lager (16.10.2026)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pololu S13V10F5 5 V/1 A Step-Up/Down</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="E2">
+        <f>C2*D2</f>
+        <v/>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/pololu-s13v10f5-5v-1a-step-up-step-down-converter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Regensensor LM393 (digital+analog)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E3">
+        <f>C3*D3</f>
+        <v/>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/regensensor-mit-digitalem-und-analogem-ausgang</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Schiebeschalter 8,6×4,3×4 mm (C&amp;K OS102011MS2QN1-Bauform)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E4">
+        <f>C4*D4</f>
+        <v/>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/schiebeschalter-printmontage-on-on-2-stellig-8.6x4.3x4mm-gerade</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BC547B NPN TO-92</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E5">
+        <f>C5*D5</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/bc547b-bipolarer-transistor-npn-45v-100ma-to-92-3-pin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Widerstand 470 Ω 1/4 W 1 %</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E6">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/metallschichtwiderstand-470-0-ohm-1-4w-1-0207-axial-durchsteckmontage</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Widerstand 4,7 kΩ 1/4 W 1 %</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E7">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/metallschichtwiderstand-4-7-kohm-1-4w-1-0207-axial-durchsteckmontage</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Widerstand 47 kΩ 1/4 W 1 % (Basis-GND, Gate Q2)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E8">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/metallschichtwiderstand-47-0-kohm-1-4w-1-0207-axial-durchsteckmontage</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Widerstand 10 kΩ 1/4 W 1 % (2× Akku-Teiler, 1× Gate Q1)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E9">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/metallschichtwiderstand-10-0-kohm-1-4w-1-0207-axial-durchsteckmontage</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Elko 470 µF/25 V radial</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E10">
+        <f>C10*D10</f>
+        <v/>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/elektrolytkondensator-470-f-25v-1050c-1-radial-tht</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SMD-Adapter SOT-23 (für AO3401A)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E11">
+        <f>C11*D11</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/smd-breakout-adapter-fuer-sot23-ssop10-msop10-10-pin-0-50mm-0-95mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Stiftleiste 1×20 RM 2,54</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E12">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/stiftleiste-1x-20-polig-rm-2-54-gerade</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lochrasterplatine doppelseitig 3×7 cm, 10 Stk (ERSATZ: 9×15 cm einseitig ist ausverkauft)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E13">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/lochrasterplatine-doppelseitig-3x7cm-10-stueck</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Vierlingslitze 4×0,14 mm², 5 m</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E14">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/vierlingslitze-isoliert-4x0-14mm-5m-farbe-blau-gelb-rot-gruen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Schrumpfschlauch-Set 100-tlg. schwarz</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E15">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/schrumpfschlauch-set-100-teilig-in-sortimentsbox-schwarz</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TESA doppelseitig 10 m × 12 mm</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="E16">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>begrenzt lagernd</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/tesa-doppelseitiges-klebeband-10m-x-12mm-transparent-pp-traeger-loesungsmittelfrei</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kabelbinder 100×2,5 mm, 100 Stk</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E17">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>auf Lager</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.berrybase.de/kabelbinder-uv-bestaendig-nylon-100-stueck/farbe-transparent/masse-100x2-5mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Reichelt</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>P-MOSFET AO3401A SOT-23 (1 Ersatz)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E18">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>auf Lager, 1–2 Werktage</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.reichelt.de/de/de/shop/produkt/mosfet_p-ch_-30v_-4a_0_041r_sot-23-166486</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>openelab.de</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Micro SD Sniffer TF Adapter Board (optional)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="E19">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>verfügbar; ggf. Versand aus China 10–20 Tage</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://openelab.de/products/micro-sd-sniffe-tf-adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Berrybase Summe</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20">
+        <f>SUMIF(A2:A19,"Berrybase",E2:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Versand: 4,95 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Reichelt Summe</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21">
+        <f>SUMIF(A2:A19,"Reichelt",E2:E19)</f>
+        <v/>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Versand: 5,95 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>openelab.de Summe</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22">
+        <f>SUMIF(A2:A19,"openelab.de",E2:E19)</f>
+        <v/>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Versand: laut Kasse</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bestellliste: Silikonmatte auf B0DS1VRH9Z (1 mm, 70x50, schwarz, 12,49 €) umgestellt
</commit_message>
<xml_diff>
--- a/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
+++ b/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
@@ -845,12 +845,12 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>FICOFISE Silikonmatte 40x30 cm</t>
+          <t>YYBYEU Silikonmatte 70x50 cm, 1 mm, schwarz</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.de/dp/B0GVNMS4DZ</t>
+          <t>https://www.amazon.de/dp/B0DS1VRH9Z</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -859,16 +859,16 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>7.59</v>
+        <v>12.49</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>1 Matte</t>
+          <t>1 Matte 70×50 cm</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>1,2 mm dick (Soll 1–1,5 mm)</t>
+          <t>1 mm dick, Versand Amazon, auf Lager (16.10.26). Alt.: B0B11N653N LEOBRO 1,3 mm 15,99 €; B0GVNMS4DZ 1,2 mm 7,59 €</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
@@ -1902,6 +1902,9 @@
       <c r="J45" s="2" t="n"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2766,7 +2769,6 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2799,7 +2801,6 @@
           <t>ja</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2945,7 +2946,6 @@
           <t>Bester Mix</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Amazon ohne Schrauben/Füße 69,52 + Berrybase 31,97 + 0,60 + Reichelt 6,46 + alleschrauben 5,82</t>
@@ -2954,7 +2954,6 @@
       <c r="F11" t="n">
         <v>114.37</v>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>+ Versand alleschrauben; bisher 139,99 €</t>

</xml_diff>

<commit_message>
Doku: microSD-Sniffer gestrichen (passt nicht ins Gehäuse)
SD-Slot zeigt zur Frontwand (ca. 3,5 mm Luft); Sniffer würde ~35–40 mm
herausstehen. GPIO18/19/23 direkt an den SD-Slot löten. Bestellsumme
Empfohlen auf 119,27 € + Versand alleschrauben korrigiert.
</commit_message>
<xml_diff>
--- a/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
+++ b/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
@@ -931,7 +931,7 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="5" t="n">
-        <v>101.56</v>
+        <v>106.46</v>
       </c>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
@@ -1832,24 +1832,24 @@
           <t>microSD-Sniffer</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C42" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>AliExpress / openelab.de (ca. 5,95 €, nicht geprüft)</t>
+          <t>nicht bestellen</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>auf Amazon.de kein Angebot gefunden; ohne Sniffer an die SD-Slot-Pads löten</t>
+          <t>nicht bestellen, passt nicht. SD-Slot zeigt zur Frontwand (nur ca. 3,5 mm Luft); Sniffer würde ca. 35–40 mm herausstehen. GPIO18/19/23 direkt an den SD-Slot löten.</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>EMPFOHLEN: A + D + Reichelt (inkl. Versand)</t>
+          <t>EMPFOHLEN: Amazon Pflicht ohne Schrauben/Füße + Berrybase inkl. Füße + Reichelt + alleschrauben (ohne Sniffer)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
@@ -1877,11 +1877,15 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="5" t="n">
-        <v>137.79</v>
+        <v>119.27</v>
       </c>
       <c r="H44" s="2" t="n"/>
       <c r="I44" s="2" t="n"/>
-      <c r="J44" s="2" t="n"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>+ Versand alleschrauben</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr"/>
@@ -2516,14 +2520,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Micro SD Sniffer TF Adapter Board (optional)</t>
+          <t>Micro SD Sniffer TF Adapter Board – NICHT BESTELLEN (passt nicht)</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
       <c r="E19">
         <f>C19*D19</f>
@@ -2531,7 +2535,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>verfügbar; ggf. Versand aus China 10–20 Tage</t>
+          <t>nicht bestellen, passt nicht. SD-Slot zeigt zur Frontwand (nur ca. 3,5 mm Luft); Sniffer würde ca. 35–40 mm herausstehen. GPIO18/19/23 direkt an den SD-Slot löten.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2575,7 +2579,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>openelab.de Summe</t>
+          <t>openelab.de Summe (Sniffer gestrichen)</t>
         </is>
       </c>
       <c r="E22">
@@ -2584,7 +2588,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Versand: laut Kasse</t>
+          <t>nicht bestellen</t>
         </is>
       </c>
     </row>
@@ -2948,15 +2952,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Amazon ohne Schrauben/Füße 69,52 + Berrybase 31,97 + 0,60 + Reichelt 6,46 + alleschrauben 5,82</t>
+          <t>Amazon ohne Schrauben/Füße 74,42 (Matte 12,49) + Berrybase 31,97 + 0,60 + Reichelt 6,46 + alleschrauben 5,82</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>114.37</v>
+        <v>119.27</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>+ Versand alleschrauben; bisher 139,99 €</t>
+          <t>+ Versand alleschrauben; Sniffer gestrichen (passt nicht)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Doku: tatsächliche Bestellung 16.10.2026 (122,13 €)
Amazon 69,52 / Berrybase 35,46 / alleschrauben 10,35 / Reichelt 6,80.
Neues Blatt und Bestellung_HydroDesk_16-10-2026.xlsx; Vorkalkulation Spalte Tatsächlich.
microSD-Sniffer und PLA nicht bestellt.
</commit_message>
<xml_diff>
--- a/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
+++ b/doku/Amazon_Bestellliste_HydroDesk_V4.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amazon-Bestellliste" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Andere Shops" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergleich Berrybase" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tatsächliche Bestellung" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00 &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +42,20 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,8 +67,23 @@
         <fgColor rgb="001F6FB2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,11 +91,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -83,6 +126,18 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2967,4 +3022,916 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Tatsächliche Bestellung HydroDesk Base – 16.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Gesamt 122,13 € (4 Belege). microSD-Sniffer und PLA nicht bestellt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Bestellnummer</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Produktname</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Menge</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Summe (€)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Hinweis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>303-9574488-4297123</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Fastsaw CYD ESP32-2432S028R 2,8" Touch TFT ILI9341 (Entwicklungsboard)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>303-9574488-4297123</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>TC4056 USB-C Lademodul mit Schutz (10er-Pack)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>303-9574488-4297123</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>DIYmalls Wägezelle 5 kg + HX711</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>303-9574488-4297123</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>FUNIANMAOYI Silikonmatte 40×30 cm, 1,2 mm (rutschfest)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="F8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>303-9574488-4297123</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>EEMB LP103454 LiPo 3,7 V 2000 mAh mit JST-PH</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>303-9574488-4297123</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>BTF-LIGHTING WS2812B FCOB COB-LED-Streifen 1 m, 160 LEDs/m, 5 mm</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>303-9574488-4297123</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Versand (frei)</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Summe Amazon</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="13" t="n">
+        <v>69.52</v>
+      </c>
+      <c r="F12" s="12" t="n"/>
+    </row>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>TESA Doppelseitiges Klebeband 10 m × 12 mm, transparent, PP-Träger, lösungsmittelfrei</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>BC547B – Bipolarer Transistor, NPN, 45 V, 100 mA, TO-92, 3-pin</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Vierlingslitze isoliert, 4×0,14 mm, 5 m – Farbe: blau, gelb, rot, grün</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Elektrolytkondensator, 470 µF, 25 V, 105 °C, ±1 %, radial, THT</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>FIX&amp;FASTEN Selbstklebender Fuß, rund, Ø oben 9,5 / unten 10 mm, Höhe 4,5 mm, Gummi, schwarz</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Metallschichtwiderstand, 10,0 kΩ, 1/4 W, ±1 %, 0207, axial</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Metallschichtwiderstand, 470,0 Ω, 1/4 W, ±1 %, 0207, axial</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F20" s="9" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Metallschichtwiderstand, 47,0 kΩ, 1/4 W, ±1 %, 0207, axial</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Metallschichtwiderstand, 4,7 kΩ, 1/4 W, ±1 %, 0207, axial</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Lochrasterplatine, doppelseitig, 3×7 cm, 10 Stück</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Stiftleiste, 1×20-polig, RM 2,54, gerade</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Pololu S13V10F5 5 V, 1 A Step-Up/Step-Down Converter</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="F25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Regensensor mit digitalem und analogem Ausgang</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F26" s="9" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Schiebeschalter, Printmontage, ON-ON, 2-stellig, 8,6×4,3×4 mm, gerade</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>SMD Breakout Adapter für SOT23 / SSOP10 / MSOP10, 10 Pin, 0,50 mm / 0,95 mm</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Kabelbinder, UV-beständig, Nylon, 100 Stück (100×2,5 mm, transparent)</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Schrumpfschlauch-Set, 100-teilig in Sortimentsbox, schwarz</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Berrybase</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>1086360</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Versand DHL Paket</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="F31" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Summe Berrybase</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="13" t="n">
+        <v>35.46</v>
+      </c>
+      <c r="F32" s="12" t="n"/>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>alleschrauben.de</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>FASTON</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Senkkopfschrauben M3×12 mit Innensechskant DIN 7991, Edelstahl A2</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>alleschrauben.de</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>FASTON</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Senkkopfschrauben M4×10 mit Innensechskant DIN 7991, Edelstahl A2</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="10" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>alleschrauben.de</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>FASTON</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Senkkopfschrauben M5×12 mit Innensechskant DIN 7991, Edelstahl A2</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="10" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>alleschrauben.de</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>FASTON</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Versand</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F37" s="9" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>Summe alleschrauben.de</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n"/>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="13" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="F38" s="12" t="n"/>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Reichelt</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>AO3401A</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>MOSFET P-CH −30 V / −4 A, 0,041 Ω, SOT-23 (AO3401A)</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="10" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F40" s="9" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>Reichelt</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>AO3401A</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Versand DHL</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="F41" s="9" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>Summe Reichelt</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="13" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F42" s="12" t="n"/>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>GESAMT</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="n"/>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>69,52 + 35,46 + 10,35 + 6,80</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="n"/>
+      <c r="E44" s="15" t="n">
+        <v>122.13</v>
+      </c>
+      <c r="F44" s="14" t="n"/>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Nicht bestellt: microSD-Sniffer (passt nicht), PLA (Schule/Betrieb).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A46:F46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>